<commit_message>
feat: add period-based A00 quantity forecasts
</commit_message>
<xml_diff>
--- a/resources/a00-new-project-template.xlsx
+++ b/resources/a00-new-project-template.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dharmamanufacturing.sharepoint.com/sites/DharmaElectrindoManufacturing/Shared Documents/Marketing/Share_SAD/DZAKKI/00. DZAKKI/2025/A00/PT. TOYO DENSO INDONESIA/BRP RYKER/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsz\Costing-System\Development\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="267" documentId="13_ncr:1_{023F1DB3-E6B2-439B-ADE2-69CA69ED128C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1FFD9FD-9E23-41A6-BF70-07DE5777112A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C34C00A8-C57E-4F0A-9802-7DB8D5353FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A00" sheetId="2" r:id="rId1"/>
     <sheet name="LAMPIRAN ASSY" sheetId="3" r:id="rId2"/>
+    <sheet name="LAMPIRAN ASSY (2)" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="79">
   <si>
     <t>NEW PROJECT
 DECLARATION</t>
@@ -274,6 +275,24 @@
   </si>
   <si>
     <t>W39801</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Assy No</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>KY A</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>LAMPIRAN FORECAST QUANTITY</t>
   </si>
 </sst>
 </file>
@@ -619,7 +638,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -738,6 +757,81 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -813,9 +907,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -831,18 +922,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -852,49 +934,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -906,35 +949,29 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2415,6 +2452,262 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>146907</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>5582</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>126936</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>96233</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="LOGO DP">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9200F6C-176A-4B4D-A46D-553B34CB39F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="394557" y="196082"/>
+          <a:ext cx="722979" cy="452601"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+          <a:round/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>69850</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76835</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>143510</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B97516E-E18B-4433-903B-67172BFDB911}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="317500" y="629285"/>
+          <a:ext cx="873125" cy="428625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="500" b="1"/>
+            <a:t>PT. DHARMA ELECTRINDO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="500" b="1"/>
+            <a:t>MANUFACTURING</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>146907</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>5582</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>126936</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>96233</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="LOGO DP">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D635F30D-B878-482E-B2C6-05D64941B003}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="394557" y="205607"/>
+          <a:ext cx="722979" cy="452601"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+          <a:round/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>69850</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76835</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>143510</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BBCF0D0-D0DD-40FA-9A7E-462F2D945EBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="317500" y="638810"/>
+          <a:ext cx="873125" cy="428625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="500" b="1"/>
+            <a:t>PT. DHARMA ELECTRINDO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="500" b="1"/>
+            <a:t>MANUFACTURING</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2719,85 +3012,85 @@
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="E2" s="16"/>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="43" t="s">
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="44"/>
-      <c r="P2" s="45"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="70"/>
       <c r="Q2" s="22" t="s">
         <v>2</v>
       </c>
       <c r="R2" s="23"/>
-      <c r="S2" s="84" t="s">
+      <c r="S2" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="T2" s="85"/>
-      <c r="U2" s="85"/>
-      <c r="V2" s="86"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="46"/>
       <c r="W2" s="13"/>
     </row>
     <row r="3" spans="1:23" ht="14.45" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="17"/>
       <c r="E3" s="18"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="47"/>
-      <c r="P3" s="48"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="82"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="73"/>
       <c r="Q3" s="24" t="s">
         <v>3</v>
       </c>
       <c r="R3" s="12"/>
-      <c r="S3" s="87">
+      <c r="S3" s="47">
         <v>45716</v>
       </c>
-      <c r="T3" s="85"/>
-      <c r="U3" s="85"/>
-      <c r="V3" s="86"/>
+      <c r="T3" s="45"/>
+      <c r="U3" s="45"/>
+      <c r="V3" s="46"/>
       <c r="W3" s="13"/>
     </row>
     <row r="4" spans="1:23" ht="14.45" customHeight="1">
       <c r="A4" s="4"/>
       <c r="B4" s="17"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="46"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="48"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="73"/>
       <c r="Q4" s="22" t="s">
         <v>4</v>
       </c>
       <c r="R4" s="23"/>
-      <c r="S4" s="88" t="s">
+      <c r="S4" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="90"/>
+      <c r="T4" s="49"/>
+      <c r="U4" s="49"/>
+      <c r="V4" s="50"/>
       <c r="W4" s="13"/>
     </row>
     <row r="5" spans="1:23" ht="14.45" customHeight="1">
@@ -2806,27 +3099,27 @@
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="20"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="60"/>
-      <c r="N5" s="49"/>
-      <c r="O5" s="50"/>
-      <c r="P5" s="51"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="74"/>
+      <c r="O5" s="75"/>
+      <c r="P5" s="76"/>
       <c r="Q5" s="25" t="s">
         <v>5</v>
       </c>
       <c r="R5" s="26"/>
-      <c r="S5" s="84" t="s">
+      <c r="S5" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="T5" s="85"/>
-      <c r="U5" s="85"/>
-      <c r="V5" s="86"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
       <c r="W5" s="13"/>
     </row>
     <row r="6" spans="1:23">
@@ -2896,7 +3189,7 @@
       <c r="J12" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K12" s="100" t="s">
+      <c r="K12" s="41" t="s">
         <v>66</v>
       </c>
       <c r="L12" s="21"/>
@@ -2950,7 +3243,7 @@
       <c r="J14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K14" s="105" t="s">
+      <c r="K14" s="43" t="s">
         <v>72</v>
       </c>
       <c r="L14" s="21"/>
@@ -2977,11 +3270,11 @@
       <c r="J15" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="91">
+      <c r="K15" s="51">
         <v>1250</v>
       </c>
-      <c r="L15" s="92"/>
-      <c r="M15" s="92"/>
+      <c r="L15" s="52"/>
+      <c r="M15" s="52"/>
       <c r="N15" s="1" t="s">
         <v>20</v>
       </c>
@@ -3050,18 +3343,18 @@
       <c r="K21" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L21" s="103" t="s">
+      <c r="L21" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="M21" s="81"/>
-      <c r="N21" s="102" t="s">
+      <c r="M21" s="54"/>
+      <c r="N21" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="O21" s="81"/>
-      <c r="P21" s="82" t="s">
+      <c r="O21" s="54"/>
+      <c r="P21" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="Q21" s="81"/>
+      <c r="Q21" s="54"/>
       <c r="S21" s="1" t="s">
         <v>27</v>
       </c>
@@ -3079,18 +3372,18 @@
       <c r="K22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L22" s="103" t="s">
+      <c r="L22" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="M22" s="81"/>
-      <c r="N22" s="102" t="s">
+      <c r="M22" s="54"/>
+      <c r="N22" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="O22" s="81"/>
-      <c r="P22" s="82" t="s">
+      <c r="O22" s="54"/>
+      <c r="P22" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="Q22" s="81"/>
+      <c r="Q22" s="54"/>
       <c r="S22" s="1" t="s">
         <v>27</v>
       </c>
@@ -3108,18 +3401,18 @@
       <c r="K23" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L23" s="103" t="s">
+      <c r="L23" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="M23" s="81"/>
-      <c r="N23" s="102" t="s">
+      <c r="M23" s="54"/>
+      <c r="N23" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="O23" s="81"/>
-      <c r="P23" s="82" t="s">
+      <c r="O23" s="54"/>
+      <c r="P23" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="Q23" s="81"/>
+      <c r="Q23" s="54"/>
       <c r="S23" s="1" t="s">
         <v>27</v>
       </c>
@@ -3137,18 +3430,18 @@
       <c r="K24" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L24" s="103" t="s">
+      <c r="L24" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="M24" s="81"/>
-      <c r="N24" s="102" t="s">
+      <c r="M24" s="54"/>
+      <c r="N24" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="O24" s="81"/>
-      <c r="P24" s="82" t="s">
+      <c r="O24" s="54"/>
+      <c r="P24" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="Q24" s="81"/>
+      <c r="Q24" s="54"/>
       <c r="S24" s="1" t="s">
         <v>27</v>
       </c>
@@ -3166,18 +3459,18 @@
       <c r="K25" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L25" s="103" t="s">
+      <c r="L25" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="M25" s="81"/>
-      <c r="N25" s="102" t="s">
+      <c r="M25" s="54"/>
+      <c r="N25" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="O25" s="81"/>
-      <c r="P25" s="82" t="s">
+      <c r="O25" s="54"/>
+      <c r="P25" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="Q25" s="81"/>
+      <c r="Q25" s="54"/>
       <c r="S25" s="1" t="s">
         <v>27</v>
       </c>
@@ -3185,12 +3478,12 @@
     </row>
     <row r="26" spans="1:23">
       <c r="A26" s="4"/>
-      <c r="L26" s="83"/>
-      <c r="M26" s="83"/>
-      <c r="N26" s="83"/>
-      <c r="O26" s="83"/>
-      <c r="P26" s="83"/>
-      <c r="Q26" s="83"/>
+      <c r="L26" s="57"/>
+      <c r="M26" s="57"/>
+      <c r="N26" s="57"/>
+      <c r="O26" s="57"/>
+      <c r="P26" s="57"/>
+      <c r="Q26" s="57"/>
       <c r="W26" s="13"/>
     </row>
     <row r="27" spans="1:23">
@@ -3218,12 +3511,12 @@
       <c r="K29" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L29" s="71"/>
-      <c r="M29" s="73"/>
-      <c r="N29" s="78"/>
-      <c r="O29" s="79"/>
-      <c r="P29" s="80"/>
-      <c r="Q29" s="73"/>
+      <c r="L29" s="60"/>
+      <c r="M29" s="61"/>
+      <c r="N29" s="58"/>
+      <c r="O29" s="59"/>
+      <c r="P29" s="62"/>
+      <c r="Q29" s="61"/>
       <c r="S29" s="32" t="s">
         <v>27</v>
       </c>
@@ -3240,12 +3533,12 @@
       <c r="K30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L30" s="71"/>
-      <c r="M30" s="73"/>
-      <c r="N30" s="78"/>
-      <c r="O30" s="79"/>
-      <c r="P30" s="80"/>
-      <c r="Q30" s="73"/>
+      <c r="L30" s="60"/>
+      <c r="M30" s="61"/>
+      <c r="N30" s="58"/>
+      <c r="O30" s="59"/>
+      <c r="P30" s="62"/>
+      <c r="Q30" s="61"/>
       <c r="S30" s="32" t="s">
         <v>27</v>
       </c>
@@ -3262,12 +3555,12 @@
       <c r="K31" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L31" s="71"/>
-      <c r="M31" s="73"/>
-      <c r="N31" s="78"/>
-      <c r="O31" s="79"/>
-      <c r="P31" s="78"/>
-      <c r="Q31" s="79"/>
+      <c r="L31" s="60"/>
+      <c r="M31" s="61"/>
+      <c r="N31" s="58"/>
+      <c r="O31" s="59"/>
+      <c r="P31" s="58"/>
+      <c r="Q31" s="59"/>
       <c r="S31" s="32" t="s">
         <v>27</v>
       </c>
@@ -3284,12 +3577,12 @@
       <c r="K32" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L32" s="71"/>
-      <c r="M32" s="73"/>
-      <c r="N32" s="78"/>
-      <c r="O32" s="79"/>
-      <c r="P32" s="78"/>
-      <c r="Q32" s="79"/>
+      <c r="L32" s="60"/>
+      <c r="M32" s="61"/>
+      <c r="N32" s="58"/>
+      <c r="O32" s="59"/>
+      <c r="P32" s="58"/>
+      <c r="Q32" s="59"/>
       <c r="S32" s="32" t="s">
         <v>27</v>
       </c>
@@ -3306,16 +3599,16 @@
       <c r="K33" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L33" s="71"/>
-      <c r="M33" s="73"/>
-      <c r="N33" s="104" t="s">
+      <c r="L33" s="60"/>
+      <c r="M33" s="61"/>
+      <c r="N33" s="99" t="s">
         <v>71</v>
       </c>
-      <c r="O33" s="79"/>
-      <c r="P33" s="104" t="s">
+      <c r="O33" s="59"/>
+      <c r="P33" s="99" t="s">
         <v>58</v>
       </c>
-      <c r="Q33" s="79"/>
+      <c r="Q33" s="59"/>
       <c r="S33" s="32" t="s">
         <v>27</v>
       </c>
@@ -3361,7 +3654,7 @@
     </row>
     <row r="43" spans="1:23">
       <c r="A43" s="4"/>
-      <c r="S43" s="101" t="s">
+      <c r="S43" s="42" t="s">
         <v>67</v>
       </c>
       <c r="T43" s="9"/>
@@ -3375,33 +3668,33 @@
     </row>
     <row r="45" spans="1:23">
       <c r="A45" s="4"/>
-      <c r="M45" s="70" t="s">
+      <c r="M45" s="94" t="s">
         <v>34</v>
       </c>
-      <c r="N45" s="70"/>
-      <c r="O45" s="70"/>
-      <c r="P45" s="70"/>
-      <c r="Q45" s="70" t="s">
+      <c r="N45" s="94"/>
+      <c r="O45" s="94"/>
+      <c r="P45" s="94"/>
+      <c r="Q45" s="94" t="s">
         <v>35</v>
       </c>
-      <c r="R45" s="70"/>
-      <c r="S45" s="70"/>
-      <c r="T45" s="71" t="s">
+      <c r="R45" s="94"/>
+      <c r="S45" s="94"/>
+      <c r="T45" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="U45" s="72"/>
-      <c r="V45" s="73"/>
+      <c r="U45" s="95"/>
+      <c r="V45" s="61"/>
       <c r="W45" s="13"/>
     </row>
     <row r="46" spans="1:23">
       <c r="A46" s="4"/>
-      <c r="M46" s="70"/>
-      <c r="N46" s="70"/>
-      <c r="O46" s="70"/>
-      <c r="P46" s="70"/>
-      <c r="Q46" s="61"/>
-      <c r="R46" s="62"/>
-      <c r="S46" s="63"/>
+      <c r="M46" s="94"/>
+      <c r="N46" s="94"/>
+      <c r="O46" s="94"/>
+      <c r="P46" s="94"/>
+      <c r="Q46" s="86"/>
+      <c r="R46" s="87"/>
+      <c r="S46" s="88"/>
       <c r="T46" s="28"/>
       <c r="U46" s="8"/>
       <c r="V46" s="29"/>
@@ -3409,77 +3702,77 @@
     </row>
     <row r="47" spans="1:23">
       <c r="A47" s="4"/>
-      <c r="M47" s="70"/>
-      <c r="N47" s="70"/>
-      <c r="O47" s="70"/>
-      <c r="P47" s="70"/>
-      <c r="Q47" s="64"/>
-      <c r="R47" s="65"/>
-      <c r="S47" s="66"/>
+      <c r="M47" s="94"/>
+      <c r="N47" s="94"/>
+      <c r="O47" s="94"/>
+      <c r="P47" s="94"/>
+      <c r="Q47" s="89"/>
+      <c r="R47" s="63"/>
+      <c r="S47" s="90"/>
       <c r="T47" s="17"/>
       <c r="V47" s="18"/>
       <c r="W47" s="13"/>
     </row>
     <row r="48" spans="1:23">
       <c r="A48" s="4"/>
-      <c r="M48" s="70"/>
-      <c r="N48" s="70"/>
-      <c r="O48" s="70"/>
-      <c r="P48" s="70"/>
-      <c r="Q48" s="67"/>
-      <c r="R48" s="68"/>
-      <c r="S48" s="69"/>
+      <c r="M48" s="94"/>
+      <c r="N48" s="94"/>
+      <c r="O48" s="94"/>
+      <c r="P48" s="94"/>
+      <c r="Q48" s="91"/>
+      <c r="R48" s="92"/>
+      <c r="S48" s="93"/>
       <c r="T48" s="17"/>
       <c r="V48" s="18"/>
       <c r="W48" s="13"/>
     </row>
     <row r="49" spans="1:23">
       <c r="A49" s="4"/>
-      <c r="M49" s="74" t="s">
+      <c r="M49" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="N49" s="74"/>
-      <c r="O49" s="74"/>
-      <c r="P49" s="74"/>
-      <c r="Q49" s="74" t="s">
+      <c r="N49" s="64"/>
+      <c r="O49" s="64"/>
+      <c r="P49" s="64"/>
+      <c r="Q49" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="R49" s="74"/>
-      <c r="S49" s="74"/>
-      <c r="T49" s="75" t="s">
+      <c r="R49" s="64"/>
+      <c r="S49" s="64"/>
+      <c r="T49" s="96" t="s">
         <v>39</v>
       </c>
-      <c r="U49" s="76"/>
-      <c r="V49" s="77"/>
+      <c r="U49" s="97"/>
+      <c r="V49" s="98"/>
       <c r="W49" s="13"/>
     </row>
     <row r="50" spans="1:23">
       <c r="A50" s="4"/>
-      <c r="B50" s="65"/>
-      <c r="C50" s="65"/>
-      <c r="D50" s="65"/>
-      <c r="E50" s="65"/>
-      <c r="F50" s="65"/>
-      <c r="G50" s="65"/>
-      <c r="H50" s="65"/>
-      <c r="I50" s="65"/>
-      <c r="J50" s="65"/>
-      <c r="M50" s="74" t="s">
+      <c r="B50" s="63"/>
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="63"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="63"/>
+      <c r="H50" s="63"/>
+      <c r="I50" s="63"/>
+      <c r="J50" s="63"/>
+      <c r="M50" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="N50" s="74"/>
-      <c r="O50" s="74"/>
-      <c r="P50" s="74"/>
-      <c r="Q50" s="74" t="s">
+      <c r="N50" s="64"/>
+      <c r="O50" s="64"/>
+      <c r="P50" s="64"/>
+      <c r="Q50" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="R50" s="74"/>
-      <c r="S50" s="74"/>
-      <c r="T50" s="40" t="s">
+      <c r="R50" s="64"/>
+      <c r="S50" s="64"/>
+      <c r="T50" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="U50" s="41"/>
-      <c r="V50" s="42"/>
+      <c r="U50" s="66"/>
+      <c r="V50" s="67"/>
       <c r="W50" s="13"/>
     </row>
     <row r="51" spans="1:23">
@@ -3553,44 +3846,6 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="S2:V2"/>
-    <mergeCell ref="S3:V3"/>
-    <mergeCell ref="S4:V4"/>
-    <mergeCell ref="S5:V5"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="P21:Q21"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="P25:Q25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="H50:J50"/>
-    <mergeCell ref="M50:P50"/>
-    <mergeCell ref="Q50:S50"/>
     <mergeCell ref="T50:V50"/>
     <mergeCell ref="N2:P5"/>
     <mergeCell ref="F2:M5"/>
@@ -3607,6 +3862,44 @@
     <mergeCell ref="P33:Q33"/>
     <mergeCell ref="L31:M31"/>
     <mergeCell ref="N31:O31"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="H50:J50"/>
+    <mergeCell ref="M50:P50"/>
+    <mergeCell ref="Q50:S50"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="P21:Q21"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="S2:V2"/>
+    <mergeCell ref="S3:V3"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="S5:V5"/>
+    <mergeCell ref="K15:M15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3637,7 +3930,7 @@
     <col min="30" max="16384" width="3.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:23" ht="15.75" thickTop="1">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3664,86 +3957,118 @@
     </row>
     <row r="2" spans="1:23" ht="14.45" customHeight="1">
       <c r="A2" s="4"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="97"/>
-      <c r="U2" s="97"/>
-      <c r="V2" s="97"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="77" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="68" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="69"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="R2" s="23"/>
+      <c r="S2" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="46"/>
       <c r="W2" s="13"/>
     </row>
     <row r="3" spans="1:23" ht="14.45" customHeight="1">
       <c r="A3" s="4"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
-      <c r="P3" s="47"/>
-      <c r="Q3" s="12"/>
+      <c r="B3" s="17"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="82"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="R3" s="12"/>
-      <c r="S3" s="98"/>
-      <c r="T3" s="97"/>
-      <c r="U3" s="97"/>
-      <c r="V3" s="97"/>
+      <c r="S3" s="47">
+        <v>45716</v>
+      </c>
+      <c r="T3" s="45"/>
+      <c r="U3" s="45"/>
+      <c r="V3" s="46"/>
       <c r="W3" s="13"/>
     </row>
     <row r="4" spans="1:23" ht="14.45" customHeight="1">
       <c r="A4" s="4"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="99"/>
-      <c r="T4" s="99"/>
-      <c r="U4" s="99"/>
-      <c r="V4" s="99"/>
+      <c r="B4" s="17"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="73"/>
+      <c r="Q4" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="R4" s="23"/>
+      <c r="S4" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" s="49"/>
+      <c r="U4" s="49"/>
+      <c r="V4" s="50"/>
       <c r="W4" s="13"/>
     </row>
     <row r="5" spans="1:23" ht="14.45" customHeight="1">
       <c r="A5" s="4"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="47"/>
-      <c r="P5" s="47"/>
-      <c r="Q5" s="12"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="97"/>
-      <c r="T5" s="97"/>
-      <c r="U5" s="97"/>
-      <c r="V5" s="97"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="74"/>
+      <c r="O5" s="75"/>
+      <c r="P5" s="76"/>
+      <c r="Q5" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="R5" s="26"/>
+      <c r="S5" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="T5" s="45"/>
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
       <c r="W5" s="13"/>
     </row>
     <row r="6" spans="1:23">
@@ -3832,105 +4157,105 @@
     </row>
     <row r="13" spans="1:23">
       <c r="A13" s="4"/>
-      <c r="D13" s="95" t="s">
+      <c r="D13" s="103" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="95"/>
-      <c r="F13" s="95"/>
-      <c r="G13" s="95"/>
-      <c r="H13" s="95"/>
-      <c r="I13" s="95" t="s">
+      <c r="E13" s="103"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="103"/>
+      <c r="I13" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="J13" s="95"/>
-      <c r="K13" s="95"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
-      <c r="N13" s="95" t="s">
+      <c r="J13" s="103"/>
+      <c r="K13" s="103"/>
+      <c r="L13" s="103"/>
+      <c r="M13" s="103"/>
+      <c r="N13" s="103" t="s">
         <v>61</v>
       </c>
-      <c r="O13" s="95"/>
-      <c r="P13" s="95"/>
-      <c r="Q13" s="95"/>
-      <c r="R13" s="95"/>
+      <c r="O13" s="103"/>
+      <c r="P13" s="103"/>
+      <c r="Q13" s="103"/>
+      <c r="R13" s="103"/>
       <c r="W13" s="13"/>
     </row>
     <row r="14" spans="1:23">
       <c r="A14" s="4"/>
-      <c r="D14" s="93" t="s">
+      <c r="D14" s="101" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="70"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="93" t="s">
+      <c r="E14" s="94"/>
+      <c r="F14" s="94"/>
+      <c r="G14" s="94"/>
+      <c r="H14" s="94"/>
+      <c r="I14" s="101" t="s">
         <v>62</v>
       </c>
-      <c r="J14" s="70"/>
-      <c r="K14" s="70"/>
-      <c r="L14" s="70"/>
-      <c r="M14" s="70"/>
-      <c r="N14" s="94">
+      <c r="J14" s="94"/>
+      <c r="K14" s="94"/>
+      <c r="L14" s="94"/>
+      <c r="M14" s="94"/>
+      <c r="N14" s="102">
         <f>20096/24</f>
         <v>837.33333333333337</v>
       </c>
-      <c r="O14" s="94"/>
-      <c r="P14" s="94"/>
-      <c r="Q14" s="94"/>
-      <c r="R14" s="94"/>
+      <c r="O14" s="102"/>
+      <c r="P14" s="102"/>
+      <c r="Q14" s="102"/>
+      <c r="R14" s="102"/>
       <c r="W14" s="13"/>
     </row>
     <row r="15" spans="1:23">
       <c r="A15" s="4"/>
-      <c r="D15" s="93" t="s">
+      <c r="D15" s="101" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="70"/>
-      <c r="F15" s="70"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="93" t="s">
+      <c r="E15" s="94"/>
+      <c r="F15" s="94"/>
+      <c r="G15" s="94"/>
+      <c r="H15" s="94"/>
+      <c r="I15" s="101" t="s">
         <v>63</v>
       </c>
-      <c r="J15" s="70"/>
-      <c r="K15" s="70"/>
-      <c r="L15" s="70"/>
-      <c r="M15" s="70"/>
-      <c r="N15" s="94">
+      <c r="J15" s="94"/>
+      <c r="K15" s="94"/>
+      <c r="L15" s="94"/>
+      <c r="M15" s="94"/>
+      <c r="N15" s="102">
         <f t="shared" ref="N15:N16" si="0">20096/24</f>
         <v>837.33333333333337</v>
       </c>
-      <c r="O15" s="94"/>
-      <c r="P15" s="94"/>
-      <c r="Q15" s="94"/>
-      <c r="R15" s="94"/>
+      <c r="O15" s="102"/>
+      <c r="P15" s="102"/>
+      <c r="Q15" s="102"/>
+      <c r="R15" s="102"/>
       <c r="W15" s="13"/>
     </row>
     <row r="16" spans="1:23" ht="14.45" customHeight="1">
       <c r="A16" s="4"/>
-      <c r="D16" s="93" t="s">
+      <c r="D16" s="101" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="93" t="s">
+      <c r="E16" s="94"/>
+      <c r="F16" s="94"/>
+      <c r="G16" s="94"/>
+      <c r="H16" s="94"/>
+      <c r="I16" s="101" t="s">
         <v>64</v>
       </c>
-      <c r="J16" s="70"/>
-      <c r="K16" s="70"/>
-      <c r="L16" s="70"/>
-      <c r="M16" s="70"/>
-      <c r="N16" s="94">
+      <c r="J16" s="94"/>
+      <c r="K16" s="94"/>
+      <c r="L16" s="94"/>
+      <c r="M16" s="94"/>
+      <c r="N16" s="102">
         <f t="shared" si="0"/>
         <v>837.33333333333337</v>
       </c>
-      <c r="O16" s="94"/>
-      <c r="P16" s="94"/>
-      <c r="Q16" s="94"/>
-      <c r="R16" s="94"/>
+      <c r="O16" s="102"/>
+      <c r="P16" s="102"/>
+      <c r="Q16" s="102"/>
+      <c r="R16" s="102"/>
       <c r="W16" s="13"/>
     </row>
     <row r="17" spans="1:44" ht="14.45" customHeight="1">
@@ -3961,17 +4286,17 @@
     </row>
     <row r="22" spans="1:44" ht="14.45" customHeight="1">
       <c r="A22" s="4"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="96"/>
-      <c r="H22" s="96"/>
-      <c r="I22" s="96"/>
-      <c r="J22" s="96"/>
-      <c r="K22" s="96"/>
-      <c r="L22" s="96"/>
-      <c r="M22" s="96"/>
-      <c r="N22" s="96"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="100"/>
+      <c r="H22" s="100"/>
+      <c r="I22" s="100"/>
+      <c r="J22" s="100"/>
+      <c r="K22" s="100"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
       <c r="O22" s="34"/>
       <c r="P22" s="34"/>
       <c r="Q22" s="34"/>
@@ -3981,17 +4306,17 @@
     </row>
     <row r="23" spans="1:44" ht="14.45" customHeight="1">
       <c r="A23" s="4"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="96"/>
-      <c r="G23" s="96"/>
-      <c r="H23" s="96"/>
-      <c r="I23" s="96"/>
-      <c r="J23" s="96"/>
-      <c r="K23" s="96"/>
-      <c r="L23" s="96"/>
-      <c r="M23" s="96"/>
-      <c r="N23" s="96"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="100"/>
+      <c r="G23" s="100"/>
+      <c r="H23" s="100"/>
+      <c r="I23" s="100"/>
+      <c r="J23" s="100"/>
+      <c r="K23" s="100"/>
+      <c r="L23" s="100"/>
+      <c r="M23" s="100"/>
+      <c r="N23" s="100"/>
       <c r="O23" s="34"/>
       <c r="P23" s="34"/>
       <c r="Q23" s="34"/>
@@ -4001,17 +4326,17 @@
     </row>
     <row r="24" spans="1:44" ht="14.45" customHeight="1">
       <c r="A24" s="4"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="96"/>
-      <c r="G24" s="96"/>
-      <c r="H24" s="96"/>
-      <c r="I24" s="96"/>
-      <c r="J24" s="96"/>
-      <c r="K24" s="96"/>
-      <c r="L24" s="96"/>
-      <c r="M24" s="96"/>
-      <c r="N24" s="96"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="100"/>
+      <c r="G24" s="100"/>
+      <c r="H24" s="100"/>
+      <c r="I24" s="100"/>
+      <c r="J24" s="100"/>
+      <c r="K24" s="100"/>
+      <c r="L24" s="100"/>
+      <c r="M24" s="100"/>
+      <c r="N24" s="100"/>
       <c r="O24" s="34"/>
       <c r="P24" s="34"/>
       <c r="Q24" s="34"/>
@@ -4021,17 +4346,17 @@
     </row>
     <row r="25" spans="1:44">
       <c r="A25" s="4"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="96"/>
-      <c r="G25" s="96"/>
-      <c r="H25" s="96"/>
-      <c r="I25" s="96"/>
-      <c r="J25" s="96"/>
-      <c r="K25" s="96"/>
-      <c r="L25" s="96"/>
-      <c r="M25" s="96"/>
-      <c r="N25" s="96"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="100"/>
+      <c r="G25" s="100"/>
+      <c r="H25" s="100"/>
+      <c r="I25" s="100"/>
+      <c r="J25" s="100"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="100"/>
+      <c r="M25" s="100"/>
+      <c r="N25" s="100"/>
       <c r="O25" s="34"/>
       <c r="P25" s="34"/>
       <c r="Q25" s="34"/>
@@ -4237,20 +4562,6 @@
     <row r="54" spans="1:23" ht="15.75" thickTop="1"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="S2:V2"/>
-    <mergeCell ref="S3:V3"/>
-    <mergeCell ref="S4:V4"/>
-    <mergeCell ref="S5:V5"/>
-    <mergeCell ref="F2:M5"/>
-    <mergeCell ref="N2:P5"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:N25"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:N22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:N23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:N24"/>
     <mergeCell ref="D16:H16"/>
     <mergeCell ref="I16:M16"/>
     <mergeCell ref="N16:R16"/>
@@ -4263,21 +4574,672 @@
     <mergeCell ref="N15:R15"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:N25"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:N22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:N23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:N24"/>
+    <mergeCell ref="S2:V2"/>
+    <mergeCell ref="S3:V3"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="S5:V5"/>
+    <mergeCell ref="F2:M5"/>
+    <mergeCell ref="N2:P5"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B86E673-9F65-4C36-99DE-B3D14BEC8057}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AR54"/>
+  <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="9" width="3.7109375" style="1"/>
+    <col min="10" max="11" width="3.5703125" style="1" customWidth="1"/>
+    <col min="12" max="17" width="3.7109375" style="1"/>
+    <col min="18" max="18" width="3" style="1" customWidth="1"/>
+    <col min="19" max="21" width="3.7109375" style="1"/>
+    <col min="22" max="22" width="5.140625" style="1" customWidth="1"/>
+    <col min="23" max="28" width="3.7109375" style="1"/>
+    <col min="29" max="29" width="6" style="1" customWidth="1"/>
+    <col min="30" max="16384" width="3.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="15.75" thickTop="1">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="11"/>
+    </row>
+    <row r="2" spans="1:23" ht="14.45" customHeight="1">
+      <c r="A2" s="4"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="77" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="68" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="69"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="R2" s="23"/>
+      <c r="S2" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="46"/>
+      <c r="W2" s="13"/>
+    </row>
+    <row r="3" spans="1:23" ht="14.45" customHeight="1">
+      <c r="A3" s="4"/>
+      <c r="B3" s="17"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="82"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="R3" s="12"/>
+      <c r="S3" s="47">
+        <v>45716</v>
+      </c>
+      <c r="T3" s="45"/>
+      <c r="U3" s="45"/>
+      <c r="V3" s="46"/>
+      <c r="W3" s="13"/>
+    </row>
+    <row r="4" spans="1:23" ht="14.45" customHeight="1">
+      <c r="A4" s="4"/>
+      <c r="B4" s="17"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="73"/>
+      <c r="Q4" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="R4" s="23"/>
+      <c r="S4" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" s="49"/>
+      <c r="U4" s="49"/>
+      <c r="V4" s="50"/>
+      <c r="W4" s="13"/>
+    </row>
+    <row r="5" spans="1:23" ht="14.45" customHeight="1">
+      <c r="A5" s="4"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="74"/>
+      <c r="O5" s="75"/>
+      <c r="P5" s="76"/>
+      <c r="Q5" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="R5" s="26"/>
+      <c r="S5" s="44" t="s">
+        <v>6</v>
+      </c>
+      <c r="T5" s="45"/>
+      <c r="U5" s="45"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="13"/>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" s="4"/>
+      <c r="W6" s="13"/>
+    </row>
+    <row r="7" spans="1:23">
+      <c r="A7" s="4"/>
+      <c r="B7" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="W7" s="13"/>
+    </row>
+    <row r="8" spans="1:23">
+      <c r="A8" s="4"/>
+      <c r="B8" s="40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="104" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="106"/>
+      <c r="E8" s="103" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="103"/>
+      <c r="G8" s="103"/>
+      <c r="H8" s="103"/>
+      <c r="I8" s="104">
+        <v>2026</v>
+      </c>
+      <c r="J8" s="105"/>
+      <c r="K8" s="104">
+        <v>2027</v>
+      </c>
+      <c r="L8" s="105"/>
+      <c r="M8" s="104">
+        <v>2028</v>
+      </c>
+      <c r="N8" s="105"/>
+      <c r="O8" s="104">
+        <v>2029</v>
+      </c>
+      <c r="P8" s="105"/>
+      <c r="Q8" s="104">
+        <v>2030</v>
+      </c>
+      <c r="R8" s="105"/>
+      <c r="S8" s="104">
+        <v>2031</v>
+      </c>
+      <c r="T8" s="105"/>
+      <c r="U8" s="104" t="s">
+        <v>75</v>
+      </c>
+      <c r="V8" s="105"/>
+      <c r="W8" s="13"/>
+    </row>
+    <row r="9" spans="1:23">
+      <c r="A9" s="4"/>
+      <c r="B9" s="107">
+        <v>1</v>
+      </c>
+      <c r="C9" s="111" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="111"/>
+      <c r="E9" s="109" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="109"/>
+      <c r="G9" s="109"/>
+      <c r="H9" s="110"/>
+      <c r="I9" s="108">
+        <v>200</v>
+      </c>
+      <c r="J9" s="110"/>
+      <c r="K9" s="108">
+        <v>1200</v>
+      </c>
+      <c r="L9" s="110"/>
+      <c r="M9" s="108">
+        <v>1200</v>
+      </c>
+      <c r="N9" s="110"/>
+      <c r="O9" s="108">
+        <v>1200</v>
+      </c>
+      <c r="P9" s="110"/>
+      <c r="Q9" s="108">
+        <v>1200</v>
+      </c>
+      <c r="R9" s="110"/>
+      <c r="S9" s="108">
+        <v>1100</v>
+      </c>
+      <c r="T9" s="110"/>
+      <c r="U9" s="108">
+        <f>SUM(I9:T9)</f>
+        <v>6100</v>
+      </c>
+      <c r="V9" s="110"/>
+      <c r="W9" s="13"/>
+    </row>
+    <row r="10" spans="1:23">
+      <c r="A10" s="4"/>
+      <c r="W10" s="13"/>
+    </row>
+    <row r="11" spans="1:23">
+      <c r="A11" s="4"/>
+      <c r="W11" s="13"/>
+    </row>
+    <row r="12" spans="1:23">
+      <c r="A12" s="4"/>
+      <c r="W12" s="13"/>
+    </row>
+    <row r="13" spans="1:23">
+      <c r="A13" s="4"/>
+      <c r="W13" s="13"/>
+    </row>
+    <row r="14" spans="1:23">
+      <c r="A14" s="4"/>
+      <c r="W14" s="13"/>
+    </row>
+    <row r="15" spans="1:23">
+      <c r="A15" s="4"/>
+      <c r="W15" s="13"/>
+    </row>
+    <row r="16" spans="1:23" ht="14.45" customHeight="1">
+      <c r="A16" s="4"/>
+      <c r="W16" s="13"/>
+    </row>
+    <row r="17" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A17" s="4"/>
+      <c r="D17" s="33"/>
+      <c r="W17" s="13"/>
+      <c r="AR17" s="32"/>
+    </row>
+    <row r="18" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A18" s="4"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="33"/>
+      <c r="W18" s="13"/>
+    </row>
+    <row r="19" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A19" s="4"/>
+      <c r="D19" s="33"/>
+      <c r="W19" s="13"/>
+    </row>
+    <row r="20" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A20" s="4"/>
+      <c r="D20" s="33"/>
+      <c r="W20" s="13"/>
+    </row>
+    <row r="21" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A21" s="4"/>
+      <c r="W21" s="13"/>
+    </row>
+    <row r="22" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A22" s="4"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="100"/>
+      <c r="H22" s="100"/>
+      <c r="I22" s="100"/>
+      <c r="J22" s="100"/>
+      <c r="K22" s="100"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="34"/>
+      <c r="P22" s="34"/>
+      <c r="Q22" s="34"/>
+      <c r="R22" s="34"/>
+      <c r="S22" s="34"/>
+      <c r="W22" s="13"/>
+    </row>
+    <row r="23" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A23" s="4"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="100"/>
+      <c r="G23" s="100"/>
+      <c r="H23" s="100"/>
+      <c r="I23" s="100"/>
+      <c r="J23" s="100"/>
+      <c r="K23" s="100"/>
+      <c r="L23" s="100"/>
+      <c r="M23" s="100"/>
+      <c r="N23" s="100"/>
+      <c r="O23" s="34"/>
+      <c r="P23" s="34"/>
+      <c r="Q23" s="34"/>
+      <c r="R23" s="34"/>
+      <c r="S23" s="34"/>
+      <c r="W23" s="13"/>
+    </row>
+    <row r="24" spans="1:44" ht="14.45" customHeight="1">
+      <c r="A24" s="4"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="100"/>
+      <c r="G24" s="100"/>
+      <c r="H24" s="100"/>
+      <c r="I24" s="100"/>
+      <c r="J24" s="100"/>
+      <c r="K24" s="100"/>
+      <c r="L24" s="100"/>
+      <c r="M24" s="100"/>
+      <c r="N24" s="100"/>
+      <c r="O24" s="34"/>
+      <c r="P24" s="34"/>
+      <c r="Q24" s="34"/>
+      <c r="R24" s="34"/>
+      <c r="S24" s="34"/>
+      <c r="W24" s="13"/>
+    </row>
+    <row r="25" spans="1:44">
+      <c r="A25" s="4"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="100"/>
+      <c r="G25" s="100"/>
+      <c r="H25" s="100"/>
+      <c r="I25" s="100"/>
+      <c r="J25" s="100"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="100"/>
+      <c r="M25" s="100"/>
+      <c r="N25" s="100"/>
+      <c r="O25" s="34"/>
+      <c r="P25" s="34"/>
+      <c r="Q25" s="34"/>
+      <c r="R25" s="34"/>
+      <c r="S25" s="34"/>
+      <c r="W25" s="13"/>
+    </row>
+    <row r="26" spans="1:44">
+      <c r="A26" s="4"/>
+      <c r="D26" s="33"/>
+      <c r="W26" s="13"/>
+    </row>
+    <row r="27" spans="1:44">
+      <c r="A27" s="4"/>
+      <c r="W27" s="13"/>
+    </row>
+    <row r="28" spans="1:44">
+      <c r="A28" s="4"/>
+      <c r="W28" s="13"/>
+    </row>
+    <row r="29" spans="1:44">
+      <c r="A29" s="4"/>
+      <c r="W29" s="13"/>
+    </row>
+    <row r="30" spans="1:44">
+      <c r="A30" s="4"/>
+      <c r="W30" s="13"/>
+    </row>
+    <row r="31" spans="1:44">
+      <c r="A31" s="4"/>
+      <c r="W31" s="13"/>
+    </row>
+    <row r="32" spans="1:44">
+      <c r="A32" s="4"/>
+      <c r="W32" s="13"/>
+    </row>
+    <row r="33" spans="1:23">
+      <c r="A33" s="4"/>
+      <c r="W33" s="13"/>
+    </row>
+    <row r="34" spans="1:23">
+      <c r="A34" s="4"/>
+      <c r="W34" s="13"/>
+    </row>
+    <row r="35" spans="1:23">
+      <c r="A35" s="4"/>
+      <c r="W35" s="13"/>
+    </row>
+    <row r="36" spans="1:23">
+      <c r="A36" s="4"/>
+      <c r="W36" s="13"/>
+    </row>
+    <row r="37" spans="1:23">
+      <c r="A37" s="4"/>
+      <c r="W37" s="13"/>
+    </row>
+    <row r="38" spans="1:23">
+      <c r="A38" s="4"/>
+      <c r="W38" s="13"/>
+    </row>
+    <row r="39" spans="1:23">
+      <c r="A39" s="4"/>
+      <c r="W39" s="13"/>
+    </row>
+    <row r="40" spans="1:23">
+      <c r="A40" s="4"/>
+      <c r="W40" s="13"/>
+    </row>
+    <row r="41" spans="1:23">
+      <c r="A41" s="4"/>
+      <c r="W41" s="13"/>
+    </row>
+    <row r="42" spans="1:23">
+      <c r="A42" s="4"/>
+      <c r="W42" s="13"/>
+    </row>
+    <row r="43" spans="1:23">
+      <c r="A43" s="4"/>
+      <c r="W43" s="13"/>
+    </row>
+    <row r="44" spans="1:23">
+      <c r="A44" s="4"/>
+      <c r="W44" s="13"/>
+    </row>
+    <row r="45" spans="1:23">
+      <c r="A45" s="4"/>
+      <c r="W45" s="13"/>
+    </row>
+    <row r="46" spans="1:23">
+      <c r="A46" s="4"/>
+      <c r="W46" s="13"/>
+    </row>
+    <row r="47" spans="1:23">
+      <c r="A47" s="4"/>
+      <c r="W47" s="13"/>
+    </row>
+    <row r="48" spans="1:23">
+      <c r="A48" s="4"/>
+      <c r="W48" s="13"/>
+    </row>
+    <row r="49" spans="1:23">
+      <c r="A49" s="4"/>
+      <c r="W49" s="13"/>
+    </row>
+    <row r="50" spans="1:23" ht="15.75" thickBot="1">
+      <c r="A50" s="6"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
+      <c r="Q50" s="7"/>
+      <c r="R50" s="7"/>
+      <c r="S50" s="7"/>
+      <c r="T50" s="7"/>
+      <c r="U50" s="7"/>
+      <c r="V50" s="7"/>
+      <c r="W50" s="14"/>
+    </row>
+    <row r="51" spans="1:23" ht="15.75" thickTop="1">
+      <c r="A51" s="4"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="36"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="36"/>
+      <c r="I51" s="36"/>
+      <c r="J51" s="36"/>
+      <c r="K51" s="36"/>
+      <c r="L51" s="36"/>
+      <c r="M51" s="36"/>
+      <c r="N51" s="36"/>
+      <c r="O51" s="36"/>
+      <c r="P51" s="36"/>
+      <c r="Q51" s="36"/>
+      <c r="R51" s="36"/>
+      <c r="S51" s="36"/>
+      <c r="T51" s="36"/>
+      <c r="U51" s="36"/>
+      <c r="V51" s="36"/>
+      <c r="W51" s="13"/>
+    </row>
+    <row r="52" spans="1:23">
+      <c r="A52" s="4"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="36"/>
+      <c r="H52" s="36"/>
+      <c r="I52" s="36"/>
+      <c r="J52" s="36"/>
+      <c r="K52" s="36"/>
+      <c r="L52" s="36"/>
+      <c r="M52" s="36"/>
+      <c r="N52" s="36"/>
+      <c r="O52" s="36"/>
+      <c r="P52" s="36"/>
+      <c r="Q52" s="36"/>
+      <c r="R52" s="36"/>
+      <c r="S52" s="36"/>
+      <c r="T52" s="36"/>
+      <c r="U52" s="36"/>
+      <c r="V52" s="36"/>
+      <c r="W52" s="13"/>
+    </row>
+    <row r="53" spans="1:23" ht="15.75" thickBot="1">
+      <c r="A53" s="6"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+      <c r="E53" s="37"/>
+      <c r="F53" s="37"/>
+      <c r="G53" s="37"/>
+      <c r="H53" s="37"/>
+      <c r="I53" s="37"/>
+      <c r="J53" s="37"/>
+      <c r="K53" s="37"/>
+      <c r="L53" s="37"/>
+      <c r="M53" s="37"/>
+      <c r="N53" s="37"/>
+      <c r="O53" s="37"/>
+      <c r="P53" s="37"/>
+      <c r="Q53" s="37"/>
+      <c r="R53" s="37"/>
+      <c r="S53" s="37"/>
+      <c r="T53" s="37"/>
+      <c r="U53" s="37"/>
+      <c r="V53" s="37"/>
+      <c r="W53" s="14"/>
+    </row>
+    <row r="54" spans="1:23" ht="15.75" thickTop="1"/>
+  </sheetData>
+  <mergeCells count="32">
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:N25"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:N22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:N23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:N24"/>
+    <mergeCell ref="F2:M5"/>
+    <mergeCell ref="N2:P5"/>
+    <mergeCell ref="S2:V2"/>
+    <mergeCell ref="S3:V3"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="S5:V5"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c4b67fe-99c5-4878-bcae-37c580b1ef7f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="efc2e60c-9564-4f53-9379-b190dde1f02d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4516,20 +5478,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c4b67fe-99c5-4878-bcae-37c580b1ef7f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="efc2e60c-9564-4f53-9379-b190dde1f02d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3098CB38-9E1E-4F2F-A279-2EC67C8F63FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{897452E0-E1BD-47F7-9D46-86D8B676B284}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="efc2e60c-9564-4f53-9379-b190dde1f02d"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="3c4b67fe-99c5-4878-bcae-37c580b1ef7f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4554,18 +5523,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{897452E0-E1BD-47F7-9D46-86D8B676B284}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3098CB38-9E1E-4F2F-A279-2EC67C8F63FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="efc2e60c-9564-4f53-9379-b190dde1f02d"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="3c4b67fe-99c5-4878-bcae-37c580b1ef7f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>